<commit_message>
Lock Time LOM fixtures to Kyle (part_no, qty) identities.
Replace dummy PN-01 count pads with confirmed rows. Tests now fail on a wrong PN or qty, not only a wrong length. Accept catalog PNs (460200, 94560), 1004611-DWG, and named dash headers (P904225-1). Skip MAIN PLATFORM later-sheet child tables. Desktop *-LOM.xlsx was not on this VM.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/lom/1004747-1-LOM.xlsx
+++ b/tests/fixtures/lom/1004747-1-LOM.xlsx
@@ -14,35 +14,25 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>-4</t>
+          <t>-2</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>-3</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>-2</t>
+          <t>ITEM</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>PART NO</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
-        <is>
-          <t>ITEM</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>PART NO</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
         <is>
           <t>DESCRIPTION</t>
         </is>
@@ -56,39 +46,29 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>17</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6993-1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>1004810-1</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PLATE A</t>
+          <t>HOSE GUIDE</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -98,27 +78,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1004806-2</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>1004811-1</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PLATE B</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -130,39 +100,29 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>15</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1004806-1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>1004812-1</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>PLATE C</t>
+          <t>OUTER BOOM SUB-WELD</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -172,34 +132,24 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>11694-2</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>1004813-1</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>PLATE D</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -209,27 +159,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>25009-2</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>1004814-1</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>PLATE E</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -241,32 +181,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>32259-1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>1004815-1</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>PLATE F</t>
+          <t>RETAINER BAR, HOSE</t>
         </is>
       </c>
     </row>
@@ -278,32 +208,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1004738-1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>1004816-1</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>PLATE G</t>
+          <t>TOP STIFFENER, OUTER BOOM</t>
         </is>
       </c>
     </row>
@@ -315,32 +235,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1004739-1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>1004817-1</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>PLATE H</t>
+          <t>BOTTOM STIFFENER, OUTER BOOM</t>
         </is>
       </c>
     </row>
@@ -352,32 +262,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1004711-1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>1004818-1</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>PLATE I</t>
+          <t>STIFFENER, CYLINDER MOUNT</t>
         </is>
       </c>
     </row>
@@ -389,32 +289,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1004741-1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>1004819-1</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>PLATE J</t>
+          <t>MASTER CYLINDER MOUNT PLATE</t>
         </is>
       </c>
     </row>
@@ -426,32 +316,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1004740-1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>1004820-1</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>GUSSET</t>
+          <t>MASTER CYLINDER MOUNT CHANNEL</t>
         </is>
       </c>
     </row>
@@ -463,32 +343,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1004773-1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>1004821-1</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>STIFFENER</t>
+          <t>CYLINDER SUPPORT</t>
         </is>
       </c>
     </row>
@@ -500,32 +370,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1004743-1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>1004822-1</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>PAD</t>
+          <t>CYLINDER ANCHOR</t>
         </is>
       </c>
     </row>
@@ -537,32 +397,103 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1004744-2</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>1004823-1</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>CLIP</t>
+          <t>BRACE, OUTER BOOM SIDE</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>1004744-1</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>BRACE, OUTER BOOM SIDE</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>1004737-1</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>PIVOT SUPPORT PLATE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>25060-6</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>TUBE, PIVOT</t>
         </is>
       </c>
     </row>
@@ -598,22 +529,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1004810-1</t>
+          <t>6993-1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>PLATE A</t>
+          <t>HOSE GUIDE</t>
         </is>
       </c>
     </row>
@@ -625,17 +556,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1004811-1</t>
+          <t>1004806-1</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>PLATE B</t>
+          <t>OUTER BOOM SUB-WELD</t>
         </is>
       </c>
     </row>
@@ -647,17 +578,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1004812-1</t>
+          <t>32259-1</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>PLATE C</t>
+          <t>RETAINER BAR, HOSE</t>
         </is>
       </c>
     </row>
@@ -669,17 +600,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1004813-1</t>
+          <t>1004738-1</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>PLATE D</t>
+          <t>TOP STIFFENER, OUTER BOOM</t>
         </is>
       </c>
     </row>
@@ -691,17 +622,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1004814-1</t>
+          <t>1004739-1</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>PLATE E</t>
+          <t>BOTTOM STIFFENER, OUTER BOOM</t>
         </is>
       </c>
     </row>
@@ -713,17 +644,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1004815-1</t>
+          <t>1004711-1</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>PLATE F</t>
+          <t>STIFFENER, CYLINDER MOUNT</t>
         </is>
       </c>
     </row>
@@ -735,17 +666,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1004816-1</t>
+          <t>1004741-1</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>PLATE G</t>
+          <t>MASTER CYLINDER MOUNT PLATE</t>
         </is>
       </c>
     </row>
@@ -757,105 +688,105 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1004817-1</t>
+          <t>1004740-1</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>PLATE H</t>
+          <t>MASTER CYLINDER MOUNT CHANNEL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1004818-1</t>
+          <t>1004773-1</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>PLATE I</t>
+          <t>CYLINDER SUPPORT</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1004819-1</t>
+          <t>1004743-1</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>PLATE J</t>
+          <t>CYLINDER ANCHOR</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1004820-1</t>
+          <t>1004744-2</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>GUSSET</t>
+          <t>BRACE, OUTER BOOM SIDE</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1004821-1</t>
+          <t>1004744-1</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>STIFFENER</t>
+          <t>BRACE, OUTER BOOM SIDE</t>
         </is>
       </c>
     </row>
@@ -867,39 +798,39 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1004822-1</t>
+          <t>1004737-1</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>PAD</t>
+          <t>PIVOT SUPPORT PLATE</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1004823-1</t>
+          <t>25060-6</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>CLIP</t>
+          <t>TUBE, PIVOT</t>
         </is>
       </c>
     </row>

</xml_diff>